<commit_message>
add test for non-content cells (e.g. styled and merged cells)
</commit_message>
<xml_diff>
--- a/Source/Test/Data/RecursiveLoopTest(2Loop).xlsx
+++ b/Source/Test/Data/RecursiveLoopTest(2Loop).xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28227"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\work\【業務用フォルダ】\Codeer.LowCode.Blazor\【ExcelReportPDFgit】\Source\Test\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Temp\Excel.Report.PDF\Source\Test\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6454BB40-0474-4D5C-901B-D3F67E8023D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2331453-0C88-4621-8F7A-06A1991F6A14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1900" yWindow="1900" windowWidth="14400" windowHeight="7270" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="30555" yWindow="3435" windowWidth="11970" windowHeight="10170" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -55,13 +55,13 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Yu Gothic"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="6"/>
-      <name val="Yu Gothic"/>
+      <name val="Calibri"/>
       <family val="3"/>
       <charset val="128"/>
       <scheme val="minor"/>
@@ -74,12 +74,24 @@
       <charset val="128"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -94,13 +106,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="49" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="標準" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -378,36 +391,35 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B10"/>
-  <sheetFormatPr defaultColWidth="4.58203125" defaultRowHeight="13"/>
+  <dimension ref="A1:D3"/>
+  <sheetFormatPr defaultColWidth="4.5703125" defaultRowHeight="13.5"/>
   <cols>
-    <col min="1" max="1" width="32.75" style="1" customWidth="1"/>
-    <col min="2" max="16384" width="4.58203125" style="1"/>
+    <col min="1" max="1" width="32.7109375" style="1" customWidth="1"/>
+    <col min="2" max="16384" width="4.5703125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:4">
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:4">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>1</v>
       </c>
+      <c r="D2" s="2"/>
     </row>
-    <row r="3" spans="1:2">
+    <row r="3" spans="1:4">
       <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="10" spans="1:2">
-      <c r="A10" s="2"/>
+      <c r="D3" s="3"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1"/>

</xml_diff>